<commit_message>
planilha referente a JAN2, FEV, MAR e ABR1
</commit_message>
<xml_diff>
--- a/banco de horas.xlsx
+++ b/banco de horas.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
   <si>
     <t>Filial</t>
   </si>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t>OBS</t>
-  </si>
-  <si>
-    <t>VERIFICAR HORÁRIO DA VOLTA</t>
   </si>
   <si>
     <t>RETORNO NO HORÁRIO NORMAL 17:00</t>
@@ -290,41 +287,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <name val="Courier New"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <b val="0"/>
@@ -543,17 +506,43 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
         </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <name val="Courier New"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
   </dxfs>
@@ -570,25 +559,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="A1:L29" totalsRowShown="0" dataDxfId="3" headerRowBorderDxfId="15" tableBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="A1:L29" totalsRowShown="0" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13">
   <autoFilter ref="A1:L29">
     <filterColumn colId="4">
-      <colorFilter dxfId="1"/>
+      <colorFilter dxfId="12"/>
     </filterColumn>
   </autoFilter>
   <tableColumns count="12">
-    <tableColumn id="1" name="Filial" dataDxfId="14"/>
-    <tableColumn id="2" name="Matricula" dataDxfId="13"/>
-    <tableColumn id="3" name="Nome" dataDxfId="12"/>
-    <tableColumn id="4" name="Saldo Anterior" dataDxfId="11"/>
-    <tableColumn id="5" name="Data" dataDxfId="10"/>
-    <tableColumn id="6" name="Evento" dataDxfId="9"/>
-    <tableColumn id="7" name="Apontamento" dataDxfId="8"/>
-    <tableColumn id="8" name="Debito" dataDxfId="7"/>
-    <tableColumn id="9" name="Credito" dataDxfId="6"/>
-    <tableColumn id="10" name="Saldo" dataDxfId="5"/>
-    <tableColumn id="11" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" name="OBS" dataDxfId="2"/>
+    <tableColumn id="1" name="Filial" dataDxfId="11"/>
+    <tableColumn id="2" name="Matricula" dataDxfId="10"/>
+    <tableColumn id="3" name="Nome" dataDxfId="9"/>
+    <tableColumn id="4" name="Saldo Anterior" dataDxfId="8"/>
+    <tableColumn id="5" name="Data" dataDxfId="7"/>
+    <tableColumn id="6" name="Evento" dataDxfId="6"/>
+    <tableColumn id="7" name="Apontamento" dataDxfId="5"/>
+    <tableColumn id="8" name="Debito" dataDxfId="4"/>
+    <tableColumn id="9" name="Credito" dataDxfId="3"/>
+    <tableColumn id="10" name="Saldo" dataDxfId="2"/>
+    <tableColumn id="11" name="Status" dataDxfId="1"/>
+    <tableColumn id="12" name="OBS" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1046,7 +1035,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -1524,7 +1513,7 @@
         <v>16</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -1578,7 +1567,7 @@
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
@@ -1700,7 +1689,7 @@
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -1720,7 +1709,7 @@
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
       <c r="L27" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -1740,26 +1729,28 @@
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
       <c r="L28" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="9">
+        <v>45036</v>
+      </c>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="2">
-        <v>45036</v>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>